<commit_message>
Handle isolated sensor outliers and clip temps
Add detection and correction for isolated faulty temperature sensors (T_data_i_1/2/3): if a sensor differs from both neighbors by >50 it is replaced by the neighbors' mean (integer division). Use numpy import, clip all T_ columns to the range [0, 1200] instead of dropping rows with out-of-range values, and only drop true NaNs. Add post-cleaning diagnostic prints (head and min/max stats). Also update Planning_previsionnel.xlsx (binary file changed).
</commit_message>
<xml_diff>
--- a/Planning_previsionnel.xlsx
+++ b/Planning_previsionnel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antoi\OneDrive\Documents\S8\Projet_Synthese_I4.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED3F8087-B2B8-45F3-8233-2615C115B9A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D007D7A-14B6-4231-AA1A-F2D11102BD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{C6E03F00-DCAA-4FE6-A67F-FD741686D31C}"/>
+    <workbookView xWindow="15" yWindow="-16320" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{C6E03F00-DCAA-4FE6-A67F-FD741686D31C}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="2" r:id="rId1"/>
@@ -490,7 +490,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -652,6 +652,7 @@
       <alignment horizontal="left" vertical="center" indent="5"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2472,8 +2473,8 @@
       <c r="O30" s="6"/>
       <c r="P30" s="6"/>
       <c r="Q30" s="6"/>
-      <c r="R30" s="30"/>
-      <c r="S30" s="6"/>
+      <c r="R30" s="63"/>
+      <c r="S30" s="30"/>
       <c r="T30" s="6"/>
       <c r="U30" s="14"/>
       <c r="V30" s="14"/>

</xml_diff>

<commit_message>
Update XGBoost script and add tuned model
Update XGBoost_qualitePrecedentes script to use only quality lags 1-2 and apply the best Optuna-tuned hyperparameters (updated n_estimators, learning_rate, max_depth, subsample, colsample_bytree, min_child_weight, gamma, regularization, etc.). Stop printing best_iteration, improve formatting, adjust lag feature reporting, and save the trained model via joblib. Rename scripts/XGBoost/XGBoost_optuna.py to XGBoost_Hyperparametres.py. Add a serialized model artifact (scripts/Autres/xgboost_model.pkl) and move fig_XGBoost_lags.png into figures/ while removing an obsolete autocorrelation image. Also include a small README MAE note update and a change to Planning_previsionnel.xlsx.
</commit_message>
<xml_diff>
--- a/Planning_previsionnel.xlsx
+++ b/Planning_previsionnel.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D007D7A-14B6-4231-AA1A-F2D11102BD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15" yWindow="-16320" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{C6E03F00-DCAA-4FE6-A67F-FD741686D31C}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{C6E03F00-DCAA-4FE6-A67F-FD741686D31C}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="2" r:id="rId1"/>
@@ -567,6 +567,41 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="5"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -618,41 +653,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -991,7 +991,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="34" t="s">
         <v>35</v>
       </c>
       <c r="B1" t="s">
@@ -1045,38 +1045,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59" t="s">
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="60" t="s">
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60" t="s">
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="59" t="s">
+      <c r="O1" s="36"/>
+      <c r="P1" s="36"/>
+      <c r="Q1" s="36"/>
+      <c r="R1" s="36"/>
+      <c r="S1" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="59"/>
+      <c r="T1" s="37"/>
       <c r="U1" s="14"/>
       <c r="V1" s="14"/>
       <c r="W1" s="14"/>
@@ -1102,7 +1102,7 @@
       <c r="AQ1" s="14"/>
     </row>
     <row r="2" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="A2" s="61"/>
+      <c r="A2" s="38"/>
       <c r="B2" s="4">
         <v>46132</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>13</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="51"/>
+      <c r="C5" s="39"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -1330,7 +1330,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="10"/>
-      <c r="C6" s="52"/>
+      <c r="C6" s="40"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -1377,7 +1377,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="10"/>
-      <c r="C7" s="52"/>
+      <c r="C7" s="40"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
@@ -1424,8 +1424,8 @@
         <v>14</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="53"/>
-      <c r="D8" s="54"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="42"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -1567,8 +1567,8 @@
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
-      <c r="E11" s="55"/>
-      <c r="F11" s="56"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="44"/>
       <c r="G11" s="2"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
@@ -1614,8 +1614,8 @@
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="57"/>
-      <c r="F12" s="58"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="46"/>
       <c r="G12" s="2"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
@@ -1710,8 +1710,8 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="46"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="59"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
@@ -1757,8 +1757,8 @@
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="47"/>
-      <c r="H15" s="48"/>
+      <c r="G15" s="60"/>
+      <c r="H15" s="61"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
@@ -1900,8 +1900,8 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="6"/>
-      <c r="I18" s="49"/>
-      <c r="J18" s="35"/>
+      <c r="I18" s="62"/>
+      <c r="J18" s="48"/>
       <c r="K18" s="6"/>
       <c r="L18" s="6"/>
       <c r="M18" s="6"/>
@@ -1947,8 +1947,8 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="6"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="41"/>
+      <c r="I19" s="63"/>
+      <c r="J19" s="54"/>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
@@ -1996,8 +1996,8 @@
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="35"/>
+      <c r="K20" s="47"/>
+      <c r="L20" s="48"/>
       <c r="M20" s="11"/>
       <c r="N20" s="6"/>
       <c r="O20" s="6"/>
@@ -2043,9 +2043,9 @@
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
-      <c r="K21" s="40"/>
-      <c r="L21" s="40"/>
-      <c r="M21" s="41"/>
+      <c r="K21" s="53"/>
+      <c r="L21" s="53"/>
+      <c r="M21" s="54"/>
       <c r="N21" s="6"/>
       <c r="O21" s="6"/>
       <c r="P21" s="6"/>
@@ -2090,9 +2090,9 @@
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
-      <c r="K22" s="40"/>
-      <c r="L22" s="40"/>
-      <c r="M22" s="41"/>
+      <c r="K22" s="53"/>
+      <c r="L22" s="53"/>
+      <c r="M22" s="54"/>
       <c r="N22" s="6"/>
       <c r="O22" s="6"/>
       <c r="P22" s="6"/>
@@ -2234,10 +2234,10 @@
       <c r="K25" s="6"/>
       <c r="L25" s="6"/>
       <c r="M25" s="28"/>
-      <c r="N25" s="36"/>
-      <c r="O25" s="36"/>
-      <c r="P25" s="36"/>
-      <c r="Q25" s="37"/>
+      <c r="N25" s="49"/>
+      <c r="O25" s="49"/>
+      <c r="P25" s="49"/>
+      <c r="Q25" s="50"/>
       <c r="R25" s="6"/>
       <c r="S25" s="6"/>
       <c r="T25" s="6"/>
@@ -2281,10 +2281,10 @@
       <c r="K26" s="6"/>
       <c r="L26" s="6"/>
       <c r="M26" s="6"/>
-      <c r="N26" s="38"/>
-      <c r="O26" s="38"/>
-      <c r="P26" s="38"/>
-      <c r="Q26" s="39"/>
+      <c r="N26" s="51"/>
+      <c r="O26" s="51"/>
+      <c r="P26" s="51"/>
+      <c r="Q26" s="52"/>
       <c r="R26" s="6"/>
       <c r="S26" s="6"/>
       <c r="T26" s="6"/>
@@ -2473,7 +2473,7 @@
       <c r="O30" s="6"/>
       <c r="P30" s="6"/>
       <c r="Q30" s="6"/>
-      <c r="R30" s="63"/>
+      <c r="R30" s="35"/>
       <c r="S30" s="30"/>
       <c r="T30" s="6"/>
       <c r="U30" s="14"/>
@@ -2564,9 +2564,9 @@
       <c r="N32" s="6"/>
       <c r="O32" s="6"/>
       <c r="P32" s="6"/>
-      <c r="Q32" s="42"/>
-      <c r="R32" s="43"/>
-      <c r="S32" s="44"/>
+      <c r="Q32" s="55"/>
+      <c r="R32" s="56"/>
+      <c r="S32" s="57"/>
       <c r="T32" s="6"/>
       <c r="U32" s="14"/>
       <c r="V32" s="14"/>
@@ -11241,21 +11241,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="N25:Q26"/>
+    <mergeCell ref="K21:M22"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="G14:H15"/>
+    <mergeCell ref="I18:J19"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E11:F12"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="K20:L20"/>
     <mergeCell ref="I1:M1"/>
     <mergeCell ref="N1:R1"/>
     <mergeCell ref="S1:T1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="C5:C7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E11:F12"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="N25:Q26"/>
-    <mergeCell ref="K21:M22"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="G14:H15"/>
-    <mergeCell ref="I18:J19"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>